<commit_message>
site build 2026-10-09 07:25
</commit_message>
<xml_diff>
--- a/models/sovereigns/Saudi_Arabia_Sovereign_Model.xlsx
+++ b/models/sovereigns/Saudi_Arabia_Sovereign_Model.xlsx
@@ -647,7 +647,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -660,11 +660,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>BIS WS_CBPOL monthly series (auto-filled; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -690,7 +686,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1.8167</v>
+        <v>1.82</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -699,7 +695,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>Aug-26</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -712,11 +708,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>IMF CPI database, all items, y/y % change, monthly (auto-filled; a run's sourced point replaces it unless older)</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -747,11 +739,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -801,7 +789,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
+          <t>IMF WEO government debt; excludes PIF, SOE and giga-project debt</t>
         </is>
       </c>
     </row>
@@ -851,11 +839,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -937,11 +921,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -994,7 +974,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>Jul-26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1009,7 +989,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Gross official reserves incl. gold at national valuation, end-month (auto-filled; a run's sourced point replaces it unless older)</t>
+          <t>gross incl. gold (gold USD 0.433bn)</t>
         </is>
       </c>
     </row>
@@ -1019,16 +999,34 @@
           <t>net_reserves_usd_bn</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n"/>
+      <c r="B17" s="2" t="n">
+        <v>482.147</v>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>USD bn</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>IMF reserve template</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>09-Oct-26</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>gross net of predetermined one-year drains (USD -6.484bn)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1037,7 +1035,7 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>15.595</v>
+        <v>15.6</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1059,11 +1057,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1123,7 +1117,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>1388.676</v>
+        <v>1388.7</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1145,11 +1139,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1280,7 +1270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1294,6 +1284,11 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
@@ -1304,7 +1299,14 @@
           <t>nominal_gdp_usd_bn</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" s="2" t="n">
+        <v>1388.7</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>IMF WEO, 09-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1312,7 +1314,14 @@
           <t>real_gdp_growth_pct</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" s="2" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>IMF WEO, 09-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1320,7 +1329,8 @@
           <t>cpi_avg_pct</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1328,7 +1338,14 @@
           <t>current_account_pct_gdp</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" s="2" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>IMF WEO, 09-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1336,7 +1353,14 @@
           <t>fiscal_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>IMF WEO, 09-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1344,7 +1368,8 @@
           <t>primary_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1352,7 +1377,14 @@
           <t>gov_debt_pct_gdp</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" s="2" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>IMF WEO, 09-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1360,7 +1392,8 @@
           <t>external_debt_pct_gdp</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1368,7 +1401,8 @@
           <t>gross_reserves_usd_bn</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1376,7 +1410,8 @@
           <t>revenue_pct_gdp</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1384,7 +1419,8 @@
           <t>interest_pct_revenue</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>